<commit_message>
Catalogue sprint: dashboard + coverage map generator, offline 045 load test, blind accuracy audit
- tools/dashboard.py: DASHBOARD.md, COVERAGE.md, coverage.csv from engine output only;
  directly verified counts human checks/physical/official page reads, never snippets
- tools/offline_load_test.mjs: replays migrations + 045 on PGlite and loads a run as the
  API does; pilot (124 candidates, 668 evidence) and full run (1,246 / 8,510) both load,
  constraint checks pass, pins table untouched
- blind audit: 83% of sampled candidates confirmed, 8% wrong/mis-structured, 8% unconfirmed
- worklist/pilot tools moved into the engine; set names fixed in checklists
- 35 engine tests pass

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EJKpUzadfBGAwYjvdRwUui
</commit_message>
<xml_diff>
--- a/docs/research/catalogue-sprint/pilot-dsuk-high/pilot_dsuk_high_checklist.xlsx
+++ b/docs/research/catalogue-sprint/pilot-dsuk-high/pilot_dsuk_high_checklist.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="162">
   <si>
     <t>Measure</t>
   </si>
@@ -173,6 +173,105 @@
     <t>dsuk/2026/spider-man-hulk-brand-new-day-lr-pin</t>
   </si>
   <si>
+    <t>Ducks of Disney Mystery Pin Pouch</t>
+  </si>
+  <si>
+    <t>Disney Parks Pin Trading 25 Years Mystery Pin Set</t>
+  </si>
+  <si>
+    <t>Stitch 626 Day 2025 Limited Release Mystery Pin Set</t>
+  </si>
+  <si>
+    <t>Experiment 626 mystery pin set (626 Day 2026)</t>
+  </si>
+  <si>
+    <t>UK: Valentine's Day Limited Release Mystery Pin Set | AU: Disney Valentine's Day 2026 Mystery 2-Piece Pin Blind Pack</t>
+  </si>
+  <si>
+    <t>The Muppets Haunted Mansion Puzzle Piece Limited Edition Mystery Pin</t>
+  </si>
+  <si>
+    <t>Mickey's Christmas Carol 24-Day Advent Calendar Mystery Pin Set 2024</t>
+  </si>
+  <si>
+    <t>Disney Halloween Limited Edition Countdown Pin Advent Calendar</t>
+  </si>
+  <si>
+    <t>Celebrating Disney Pins 25th Anniversary Limited Edition Pin Set Series, 1 of 4</t>
+  </si>
+  <si>
+    <t>Celebrating Disney Pins 25th Anniversary Limited Edition Pin Set Series, 2 of 4</t>
+  </si>
+  <si>
+    <t>Celebrating Disney Pins 25th Anniversary Limited Edition Pin Set Series, 3 of 4</t>
+  </si>
+  <si>
+    <t>Mickey and Friends Celebrating Disney Pins 25th Anniversary Limited Edition Pin Set Series, 4 of 4</t>
+  </si>
+  <si>
+    <t>Chip 'n Dale Limited Release Christmas Countdown 2024 Jumbo Pin</t>
+  </si>
+  <si>
+    <t>Disney Magical Collections (2024)</t>
+  </si>
+  <si>
+    <t>Mushu Lunar New Year 2024 Limited Release Pin</t>
+  </si>
+  <si>
+    <t>Magical Medallions (January 2024 releases)</t>
+  </si>
+  <si>
+    <t>Mickey Mouse and Santa Claus Limited Release Festive Pin 2024</t>
+  </si>
+  <si>
+    <t>Moana, Simea, Pua and Hei Hei Limited Release Pin, Moana 2</t>
+  </si>
+  <si>
+    <t>Santa Mickey Mouse Limited Edition Festive Pin 2024</t>
+  </si>
+  <si>
+    <t>Mickey Mouse and Minnie Mouse St. David's Day 2024 Limited Edition Pin</t>
+  </si>
+  <si>
+    <t>Stitch St. Patrick's Day 2025 Limited Release Slider Pin</t>
+  </si>
+  <si>
+    <t>Ariel and King Triton Father's Day 2026 Limited Release Pin</t>
+  </si>
+  <si>
+    <t>Spider-Man and Hulk Limited Release Pin, Spider-Man: Brand New Day</t>
+  </si>
+  <si>
+    <t>2025-03-12</t>
+  </si>
+  <si>
+    <t>2025-05-22</t>
+  </si>
+  <si>
+    <t>2024-09-30</t>
+  </si>
+  <si>
+    <t>2025-07-28</t>
+  </si>
+  <si>
+    <t>2025-04-01</t>
+  </si>
+  <si>
+    <t>2025-10-08</t>
+  </si>
+  <si>
+    <t>2024-01</t>
+  </si>
+  <si>
+    <t>2023-12-12</t>
+  </si>
+  <si>
+    <t>2024-02</t>
+  </si>
+  <si>
+    <t>2026-06-02</t>
+  </si>
+  <si>
     <t>official</t>
   </si>
   <si>
@@ -284,9 +383,6 @@
     <t>Daisy Duck – Mickey and Friends Celebrating Disney Pins 25th Anniversary Limited Edition Pin Set Series, 4 of 4 | Mickey Mouse; Minnie Mouse | Pluto – Mickey and Friends Celebrating Disney Pins 25th Anniversary Limited Edition Pin Set Series, 4 of 4</t>
   </si>
   <si>
-    <t>Chip 'n Dale Limited Release Christmas Countdown 2024 Jumbo Pin</t>
-  </si>
-  <si>
     <t>Belle and Chip Magical Collections Pin</t>
   </si>
   <si>
@@ -308,16 +404,10 @@
     <t>Mickey Mouse – Santa Mickey Mouse Limited Edition Festive Pin 2024</t>
   </si>
   <si>
-    <t>Mickey Mouse and Minnie Mouse St. David's Day 2024 Limited Edition Pin</t>
-  </si>
-  <si>
     <t>Stitch St. Patrick's Day 2025 Limited Release Slider Pin, Lilo &amp; Stitch</t>
   </si>
   <si>
     <t>Ariel; King Triton</t>
-  </si>
-  <si>
-    <t>Spider-Man and Hulk Limited Release Pin, Spider-Man: Brand New Day</t>
   </si>
   <si>
     <t>dsuk/2025/ducks-of-disney-mystery-pouch/baymax | dsuk/2025/ducks-of-disney-mystery-pouch/cheshire-cat | dsuk/2025/ducks-of-disney-mystery-pouch/daisy | dsuk/2025/ducks-of-disney-mystery-pouch/donald | dsuk/2025/ducks-of-disney-mystery-pouch/dumbo | dsuk/2025/ducks-of-disney-mystery-pouch/figment | dsuk/2025/ducks-of-disney-mystery-pouch/goofy | dsuk/2025/ducks-of-disney-mystery-pouch/marie | dsuk/2025/ducks-of-disney-mystery-pouch/minnie | dsuk/2025/ducks-of-disney-mystery-pouch/nemo | dsuk/2025/ducks-of-disney-mystery-pouch/pluto | dsuk/2025/ducks-of-disney-mystery-pouch/powerline | dsuk/2025/ducks-of-disney-mystery-pouch/sorcerer-mickey | dsuk/2025/ducks-of-disney-mystery-pouch/stitch | dsuk/2025/ducks-of-disney-mystery-pouch/tigger | dsuk/2025/ducks-of-disney-mystery-pouch/tinker-bell</t>
@@ -900,7 +990,10 @@
         <v>29</v>
       </c>
       <c r="E2" t="s">
-        <v>29</v>
+        <v>52</v>
+      </c>
+      <c r="F2" t="s">
+        <v>75</v>
       </c>
       <c r="G2">
         <v>16</v>
@@ -918,16 +1011,16 @@
         <v>0</v>
       </c>
       <c r="L2" t="s">
-        <v>52</v>
+        <v>85</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>53</v>
+        <v>86</v>
       </c>
       <c r="N2" t="s">
-        <v>77</v>
+        <v>110</v>
       </c>
       <c r="O2" t="s">
-        <v>101</v>
+        <v>131</v>
       </c>
     </row>
     <row r="3" spans="1:20">
@@ -944,7 +1037,7 @@
         <v>30</v>
       </c>
       <c r="E3" t="s">
-        <v>30</v>
+        <v>53</v>
       </c>
       <c r="G3">
         <v>10</v>
@@ -962,16 +1055,16 @@
         <v>0</v>
       </c>
       <c r="L3" t="s">
-        <v>52</v>
+        <v>85</v>
       </c>
       <c r="M3" s="1" t="s">
-        <v>54</v>
+        <v>87</v>
       </c>
       <c r="N3" t="s">
-        <v>78</v>
+        <v>111</v>
       </c>
       <c r="O3" t="s">
-        <v>102</v>
+        <v>132</v>
       </c>
     </row>
     <row r="4" spans="1:20">
@@ -988,7 +1081,10 @@
         <v>31</v>
       </c>
       <c r="E4" t="s">
-        <v>31</v>
+        <v>54</v>
+      </c>
+      <c r="F4" t="s">
+        <v>76</v>
       </c>
       <c r="G4">
         <v>10</v>
@@ -1006,16 +1102,16 @@
         <v>0</v>
       </c>
       <c r="L4" t="s">
-        <v>52</v>
+        <v>85</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>55</v>
+        <v>88</v>
       </c>
       <c r="N4" t="s">
-        <v>79</v>
+        <v>112</v>
       </c>
       <c r="O4" t="s">
-        <v>103</v>
+        <v>133</v>
       </c>
     </row>
     <row r="5" spans="1:20">
@@ -1032,7 +1128,7 @@
         <v>32</v>
       </c>
       <c r="E5" t="s">
-        <v>32</v>
+        <v>55</v>
       </c>
       <c r="G5">
         <v>10</v>
@@ -1050,16 +1146,16 @@
         <v>0</v>
       </c>
       <c r="L5" t="s">
-        <v>52</v>
+        <v>85</v>
       </c>
       <c r="M5" s="1" t="s">
-        <v>56</v>
+        <v>89</v>
       </c>
       <c r="N5" t="s">
-        <v>80</v>
+        <v>113</v>
       </c>
       <c r="O5" t="s">
-        <v>104</v>
+        <v>134</v>
       </c>
     </row>
     <row r="6" spans="1:20">
@@ -1076,7 +1172,7 @@
         <v>33</v>
       </c>
       <c r="E6" t="s">
-        <v>33</v>
+        <v>56</v>
       </c>
       <c r="G6">
         <v>10</v>
@@ -1094,19 +1190,19 @@
         <v>0</v>
       </c>
       <c r="L6" t="s">
-        <v>52</v>
+        <v>85</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>57</v>
+        <v>90</v>
       </c>
       <c r="N6" t="s">
-        <v>81</v>
+        <v>114</v>
       </c>
       <c r="O6" t="s">
-        <v>105</v>
+        <v>135</v>
       </c>
       <c r="T6" t="s">
-        <v>125</v>
+        <v>155</v>
       </c>
     </row>
     <row r="7" spans="1:20">
@@ -1123,7 +1219,7 @@
         <v>34</v>
       </c>
       <c r="E7" t="s">
-        <v>34</v>
+        <v>57</v>
       </c>
       <c r="G7">
         <v>10</v>
@@ -1141,16 +1237,16 @@
         <v>0</v>
       </c>
       <c r="L7" t="s">
-        <v>52</v>
+        <v>85</v>
       </c>
       <c r="M7" s="1" t="s">
-        <v>58</v>
+        <v>91</v>
       </c>
       <c r="N7" t="s">
-        <v>82</v>
+        <v>115</v>
       </c>
       <c r="O7" t="s">
-        <v>106</v>
+        <v>136</v>
       </c>
     </row>
     <row r="8" spans="1:20">
@@ -1167,7 +1263,10 @@
         <v>35</v>
       </c>
       <c r="E8" t="s">
-        <v>35</v>
+        <v>58</v>
+      </c>
+      <c r="F8" t="s">
+        <v>77</v>
       </c>
       <c r="G8">
         <v>7</v>
@@ -1185,19 +1284,19 @@
         <v>0</v>
       </c>
       <c r="L8" t="s">
-        <v>52</v>
+        <v>85</v>
       </c>
       <c r="M8" s="1" t="s">
-        <v>59</v>
+        <v>92</v>
       </c>
       <c r="N8" t="s">
-        <v>83</v>
+        <v>116</v>
       </c>
       <c r="O8" t="s">
-        <v>107</v>
+        <v>137</v>
       </c>
       <c r="T8" t="s">
-        <v>126</v>
+        <v>156</v>
       </c>
     </row>
     <row r="9" spans="1:20">
@@ -1214,7 +1313,10 @@
         <v>36</v>
       </c>
       <c r="E9" t="s">
-        <v>36</v>
+        <v>59</v>
+      </c>
+      <c r="F9" t="s">
+        <v>78</v>
       </c>
       <c r="G9">
         <v>7</v>
@@ -1232,16 +1334,16 @@
         <v>0</v>
       </c>
       <c r="L9" t="s">
-        <v>52</v>
+        <v>85</v>
       </c>
       <c r="M9" s="1" t="s">
-        <v>60</v>
+        <v>93</v>
       </c>
       <c r="N9" t="s">
-        <v>84</v>
+        <v>117</v>
       </c>
       <c r="O9" t="s">
-        <v>108</v>
+        <v>138</v>
       </c>
     </row>
     <row r="10" spans="1:20">
@@ -1258,7 +1360,7 @@
         <v>37</v>
       </c>
       <c r="E10" t="s">
-        <v>37</v>
+        <v>60</v>
       </c>
       <c r="G10">
         <v>3</v>
@@ -1276,16 +1378,16 @@
         <v>0</v>
       </c>
       <c r="L10" t="s">
-        <v>52</v>
+        <v>85</v>
       </c>
       <c r="M10" s="1" t="s">
-        <v>61</v>
+        <v>94</v>
       </c>
       <c r="N10" t="s">
-        <v>85</v>
+        <v>118</v>
       </c>
       <c r="O10" t="s">
-        <v>109</v>
+        <v>139</v>
       </c>
     </row>
     <row r="11" spans="1:20">
@@ -1302,7 +1404,10 @@
         <v>38</v>
       </c>
       <c r="E11" t="s">
-        <v>38</v>
+        <v>61</v>
+      </c>
+      <c r="F11" t="s">
+        <v>79</v>
       </c>
       <c r="G11">
         <v>3</v>
@@ -1320,16 +1425,16 @@
         <v>0</v>
       </c>
       <c r="L11" t="s">
-        <v>52</v>
+        <v>85</v>
       </c>
       <c r="M11" s="1" t="s">
-        <v>62</v>
+        <v>95</v>
       </c>
       <c r="N11" t="s">
-        <v>86</v>
+        <v>119</v>
       </c>
       <c r="O11" t="s">
-        <v>110</v>
+        <v>140</v>
       </c>
     </row>
     <row r="12" spans="1:20">
@@ -1346,7 +1451,7 @@
         <v>39</v>
       </c>
       <c r="E12" t="s">
-        <v>39</v>
+        <v>62</v>
       </c>
       <c r="G12">
         <v>3</v>
@@ -1364,16 +1469,16 @@
         <v>0</v>
       </c>
       <c r="L12" t="s">
-        <v>52</v>
+        <v>85</v>
       </c>
       <c r="M12" s="1" t="s">
-        <v>63</v>
+        <v>96</v>
       </c>
       <c r="N12" t="s">
-        <v>87</v>
+        <v>120</v>
       </c>
       <c r="O12" t="s">
-        <v>111</v>
+        <v>141</v>
       </c>
     </row>
     <row r="13" spans="1:20">
@@ -1390,7 +1495,10 @@
         <v>40</v>
       </c>
       <c r="E13" t="s">
-        <v>40</v>
+        <v>63</v>
+      </c>
+      <c r="F13" t="s">
+        <v>80</v>
       </c>
       <c r="G13">
         <v>3</v>
@@ -1408,16 +1516,16 @@
         <v>0</v>
       </c>
       <c r="L13" t="s">
-        <v>52</v>
+        <v>85</v>
       </c>
       <c r="M13" s="1" t="s">
-        <v>64</v>
+        <v>97</v>
       </c>
       <c r="N13" t="s">
-        <v>88</v>
+        <v>121</v>
       </c>
       <c r="O13" t="s">
-        <v>112</v>
+        <v>142</v>
       </c>
     </row>
     <row r="14" spans="1:20">
@@ -1434,7 +1542,7 @@
         <v>41</v>
       </c>
       <c r="E14" t="s">
-        <v>41</v>
+        <v>64</v>
       </c>
       <c r="G14">
         <v>1</v>
@@ -1452,16 +1560,16 @@
         <v>0</v>
       </c>
       <c r="L14" t="s">
-        <v>52</v>
+        <v>85</v>
       </c>
       <c r="M14" s="1" t="s">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="N14" t="s">
-        <v>89</v>
+        <v>64</v>
       </c>
       <c r="O14" t="s">
-        <v>113</v>
+        <v>143</v>
       </c>
     </row>
     <row r="15" spans="1:20">
@@ -1478,7 +1586,10 @@
         <v>42</v>
       </c>
       <c r="E15" t="s">
-        <v>42</v>
+        <v>65</v>
+      </c>
+      <c r="F15" t="s">
+        <v>81</v>
       </c>
       <c r="G15">
         <v>1</v>
@@ -1496,19 +1607,19 @@
         <v>0</v>
       </c>
       <c r="L15" t="s">
-        <v>52</v>
+        <v>85</v>
       </c>
       <c r="M15" s="1" t="s">
-        <v>66</v>
+        <v>99</v>
       </c>
       <c r="N15" t="s">
-        <v>90</v>
+        <v>122</v>
       </c>
       <c r="O15" t="s">
-        <v>114</v>
+        <v>144</v>
       </c>
       <c r="T15" t="s">
-        <v>127</v>
+        <v>157</v>
       </c>
     </row>
     <row r="16" spans="1:20">
@@ -1525,7 +1636,10 @@
         <v>42</v>
       </c>
       <c r="E16" t="s">
-        <v>42</v>
+        <v>65</v>
+      </c>
+      <c r="F16" t="s">
+        <v>81</v>
       </c>
       <c r="G16">
         <v>1</v>
@@ -1543,19 +1657,19 @@
         <v>0</v>
       </c>
       <c r="L16" t="s">
-        <v>52</v>
+        <v>85</v>
       </c>
       <c r="M16" s="1" t="s">
-        <v>67</v>
+        <v>100</v>
       </c>
       <c r="N16" t="s">
-        <v>91</v>
+        <v>123</v>
       </c>
       <c r="O16" t="s">
-        <v>115</v>
+        <v>145</v>
       </c>
       <c r="T16" t="s">
-        <v>128</v>
+        <v>158</v>
       </c>
     </row>
     <row r="17" spans="1:20">
@@ -1572,7 +1686,10 @@
         <v>43</v>
       </c>
       <c r="E17" t="s">
-        <v>43</v>
+        <v>66</v>
+      </c>
+      <c r="F17" t="s">
+        <v>82</v>
       </c>
       <c r="G17">
         <v>1</v>
@@ -1590,19 +1707,19 @@
         <v>0</v>
       </c>
       <c r="L17" t="s">
-        <v>52</v>
+        <v>85</v>
       </c>
       <c r="M17" s="1" t="s">
-        <v>68</v>
+        <v>101</v>
       </c>
       <c r="N17" t="s">
-        <v>92</v>
+        <v>124</v>
       </c>
       <c r="O17" t="s">
-        <v>116</v>
+        <v>146</v>
       </c>
       <c r="T17" t="s">
-        <v>129</v>
+        <v>159</v>
       </c>
     </row>
     <row r="18" spans="1:20">
@@ -1619,7 +1736,10 @@
         <v>44</v>
       </c>
       <c r="E18" t="s">
-        <v>44</v>
+        <v>67</v>
+      </c>
+      <c r="F18" t="s">
+        <v>81</v>
       </c>
       <c r="G18">
         <v>1</v>
@@ -1637,16 +1757,16 @@
         <v>0</v>
       </c>
       <c r="L18" t="s">
-        <v>52</v>
+        <v>85</v>
       </c>
       <c r="M18" s="1" t="s">
-        <v>69</v>
+        <v>102</v>
       </c>
       <c r="N18" t="s">
-        <v>93</v>
+        <v>125</v>
       </c>
       <c r="O18" t="s">
-        <v>117</v>
+        <v>147</v>
       </c>
     </row>
     <row r="19" spans="1:20">
@@ -1663,7 +1783,7 @@
         <v>45</v>
       </c>
       <c r="E19" t="s">
-        <v>45</v>
+        <v>68</v>
       </c>
       <c r="G19">
         <v>1</v>
@@ -1681,16 +1801,16 @@
         <v>0</v>
       </c>
       <c r="L19" t="s">
-        <v>52</v>
+        <v>85</v>
       </c>
       <c r="M19" s="1" t="s">
-        <v>70</v>
+        <v>103</v>
       </c>
       <c r="N19" t="s">
-        <v>94</v>
+        <v>126</v>
       </c>
       <c r="O19" t="s">
-        <v>118</v>
+        <v>148</v>
       </c>
     </row>
     <row r="20" spans="1:20">
@@ -1707,7 +1827,7 @@
         <v>46</v>
       </c>
       <c r="E20" t="s">
-        <v>46</v>
+        <v>69</v>
       </c>
       <c r="G20">
         <v>1</v>
@@ -1725,19 +1845,19 @@
         <v>0</v>
       </c>
       <c r="L20" t="s">
-        <v>52</v>
+        <v>85</v>
       </c>
       <c r="M20" s="1" t="s">
-        <v>71</v>
+        <v>104</v>
       </c>
       <c r="N20" t="s">
-        <v>95</v>
+        <v>127</v>
       </c>
       <c r="O20" t="s">
-        <v>119</v>
+        <v>149</v>
       </c>
       <c r="T20" t="s">
-        <v>130</v>
+        <v>160</v>
       </c>
     </row>
     <row r="21" spans="1:20">
@@ -1754,7 +1874,7 @@
         <v>47</v>
       </c>
       <c r="E21" t="s">
-        <v>47</v>
+        <v>70</v>
       </c>
       <c r="G21">
         <v>1</v>
@@ -1772,16 +1892,16 @@
         <v>0</v>
       </c>
       <c r="L21" t="s">
-        <v>52</v>
+        <v>85</v>
       </c>
       <c r="M21" s="1" t="s">
-        <v>72</v>
+        <v>105</v>
       </c>
       <c r="N21" t="s">
-        <v>96</v>
+        <v>128</v>
       </c>
       <c r="O21" t="s">
-        <v>120</v>
+        <v>150</v>
       </c>
     </row>
     <row r="22" spans="1:20">
@@ -1798,7 +1918,10 @@
         <v>48</v>
       </c>
       <c r="E22" t="s">
-        <v>48</v>
+        <v>71</v>
+      </c>
+      <c r="F22" t="s">
+        <v>83</v>
       </c>
       <c r="G22">
         <v>1</v>
@@ -1816,16 +1939,16 @@
         <v>0</v>
       </c>
       <c r="L22" t="s">
-        <v>52</v>
+        <v>85</v>
       </c>
       <c r="M22" s="1" t="s">
-        <v>73</v>
+        <v>106</v>
       </c>
       <c r="N22" t="s">
-        <v>97</v>
+        <v>71</v>
       </c>
       <c r="O22" t="s">
-        <v>121</v>
+        <v>151</v>
       </c>
     </row>
     <row r="23" spans="1:20">
@@ -1842,7 +1965,7 @@
         <v>49</v>
       </c>
       <c r="E23" t="s">
-        <v>49</v>
+        <v>72</v>
       </c>
       <c r="G23">
         <v>1</v>
@@ -1860,19 +1983,19 @@
         <v>0</v>
       </c>
       <c r="L23" t="s">
-        <v>52</v>
+        <v>85</v>
       </c>
       <c r="M23" s="1" t="s">
-        <v>74</v>
+        <v>107</v>
       </c>
       <c r="N23" t="s">
-        <v>98</v>
+        <v>129</v>
       </c>
       <c r="O23" t="s">
-        <v>122</v>
+        <v>152</v>
       </c>
       <c r="T23" t="s">
-        <v>131</v>
+        <v>161</v>
       </c>
     </row>
     <row r="24" spans="1:20">
@@ -1889,7 +2012,10 @@
         <v>50</v>
       </c>
       <c r="E24" t="s">
-        <v>50</v>
+        <v>73</v>
+      </c>
+      <c r="F24" t="s">
+        <v>84</v>
       </c>
       <c r="G24">
         <v>1</v>
@@ -1907,16 +2033,16 @@
         <v>0</v>
       </c>
       <c r="L24" t="s">
-        <v>52</v>
+        <v>85</v>
       </c>
       <c r="M24" s="1" t="s">
-        <v>75</v>
+        <v>108</v>
       </c>
       <c r="N24" t="s">
-        <v>99</v>
+        <v>130</v>
       </c>
       <c r="O24" t="s">
-        <v>123</v>
+        <v>153</v>
       </c>
     </row>
     <row r="25" spans="1:20">
@@ -1933,7 +2059,7 @@
         <v>51</v>
       </c>
       <c r="E25" t="s">
-        <v>51</v>
+        <v>74</v>
       </c>
       <c r="G25">
         <v>1</v>
@@ -1951,16 +2077,16 @@
         <v>0</v>
       </c>
       <c r="L25" t="s">
-        <v>52</v>
+        <v>85</v>
       </c>
       <c r="M25" s="1" t="s">
-        <v>76</v>
+        <v>109</v>
       </c>
       <c r="N25" t="s">
-        <v>100</v>
+        <v>74</v>
       </c>
       <c r="O25" t="s">
-        <v>124</v>
+        <v>154</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Catalogue engine: structure-check flag on multi-character pins (top audit error); refresh outputs
207 pins flagged for one-pin-vs-separate confirmation (24 in the DSUK pilot);
pilot reloads offline with all guards passing. 36 tests pass, audit clean.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EJKpUzadfBGAwYjvdRwUui
</commit_message>
<xml_diff>
--- a/docs/research/catalogue-sprint/pilot-dsuk-high/pilot_dsuk_high_checklist.xlsx
+++ b/docs/research/catalogue-sprint/pilot-dsuk-high/pilot_dsuk_high_checklist.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="172">
   <si>
     <t>Measure</t>
   </si>
@@ -38,6 +38,9 @@
     <t>exact catalogue duplicate</t>
   </si>
   <si>
+    <t>multi-character (confirm structure)</t>
+  </si>
+  <si>
     <t>sets</t>
   </si>
   <si>
@@ -482,13 +485,31 @@
     <t>dsuk/2026/spider-man-hulk-brand-new-day-lr-pin/spider-man-and-hulk</t>
   </si>
   <si>
+    <t>627: check one pin vs separate pins; angel: check one pin vs separate pins; jumba: check one pin vs separate pins; kixx: check one pin vs separate pins; leroy: check one pin vs separate pins; reuben: check one pin vs separate pins; richter: check one pin vs separate pins; sinker: check one pin vs separate pins; splodyhead: check one pin vs separate pins; yaarp: check one pin vs separate pins</t>
+  </si>
+  <si>
     <t>powerline: possible duplicate; stitch: possible duplicate; winnie-the-pooh: possible duplicate</t>
   </si>
   <si>
+    <t>bunsen-and-beaker-as-busts: check one pin vs separate pins; gonzo-and-pepe-as-servants: check one pin vs separate pins; sam-eagle-and-pops-as-ghosts: check one pin vs separate pins</t>
+  </si>
+  <si>
     <t>daisy-isabelle: variants: add a note; donald-fred: variants: add a note; goofy-marleys-ghost: variants: add a note; jiminy-cricket-ghost-of-christmas-past: variants: add a note; mickey-bob-cratchit: variants: add a note; minnie-emily-cratchit: variants: add a note; scrooge-mcduck-ebenezer-scrooge: variants: add a note</t>
   </si>
   <si>
-    <t>belle-and-chip: variants: add a note</t>
+    <t>chip-n-dale: check one pin vs separate pins</t>
+  </si>
+  <si>
+    <t>stitch-with-angel: check one pin vs separate pins</t>
+  </si>
+  <si>
+    <t>kermit-and-miss-piggy: check one pin vs separate pins</t>
+  </si>
+  <si>
+    <t>mickey-and-minnie: check one pin vs separate pins</t>
+  </si>
+  <si>
+    <t>belle-and-chip: variants: add a note, check one pin vs separate pins</t>
   </si>
   <si>
     <t>dug: variants: add a note</t>
@@ -497,10 +518,19 @@
     <t>mushu: variants: add a note</t>
   </si>
   <si>
-    <t>moana-simea-pua-heihei: variants: add a note</t>
+    <t>mickey-mouse-and-santa-claus: check one pin vs separate pins</t>
+  </si>
+  <si>
+    <t>moana-simea-pua-heihei: variants: add a note, check one pin vs separate pins</t>
   </si>
   <si>
     <t>stitch: variants: add a note</t>
+  </si>
+  <si>
+    <t>ariel-and-king-triton: check one pin vs separate pins</t>
+  </si>
+  <si>
+    <t>spider-man-and-hulk: check one pin vs separate pins</t>
   </si>
 </sst>
 </file>
@@ -845,7 +875,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -901,6 +931,14 @@
         <v>7</v>
       </c>
       <c r="B7">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8">
         <v>23</v>
       </c>
     </row>
@@ -916,64 +954,64 @@
   <sheetData>
     <row r="1" spans="1:20">
       <c r="A1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="K1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="M1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="N1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="O1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="P1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="Q1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="R1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="S1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="T1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:20">
@@ -984,16 +1022,16 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G2">
         <v>16</v>
@@ -1011,16 +1049,16 @@
         <v>0</v>
       </c>
       <c r="L2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="N2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="O2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="3" spans="1:20">
@@ -1031,13 +1069,13 @@
         <v>4</v>
       </c>
       <c r="C3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G3">
         <v>10</v>
@@ -1055,16 +1093,16 @@
         <v>0</v>
       </c>
       <c r="L3" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="M3" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="N3" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="O3" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="4" spans="1:20">
@@ -1075,16 +1113,16 @@
         <v>5</v>
       </c>
       <c r="C4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G4">
         <v>10</v>
@@ -1102,16 +1140,16 @@
         <v>0</v>
       </c>
       <c r="L4" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="N4" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="O4" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="5" spans="1:20">
@@ -1122,13 +1160,13 @@
         <v>6</v>
       </c>
       <c r="C5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G5">
         <v>10</v>
@@ -1146,16 +1184,19 @@
         <v>0</v>
       </c>
       <c r="L5" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="M5" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="N5" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="O5" t="s">
-        <v>134</v>
+        <v>135</v>
+      </c>
+      <c r="T5" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="6" spans="1:20">
@@ -1166,13 +1207,13 @@
         <v>7</v>
       </c>
       <c r="C6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G6">
         <v>10</v>
@@ -1190,19 +1231,19 @@
         <v>0</v>
       </c>
       <c r="L6" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="N6" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="O6" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="T6" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="7" spans="1:20">
@@ -1213,13 +1254,13 @@
         <v>8</v>
       </c>
       <c r="C7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G7">
         <v>10</v>
@@ -1237,16 +1278,19 @@
         <v>0</v>
       </c>
       <c r="L7" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="M7" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="N7" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="O7" t="s">
-        <v>136</v>
+        <v>137</v>
+      </c>
+      <c r="T7" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="8" spans="1:20">
@@ -1257,16 +1301,16 @@
         <v>11</v>
       </c>
       <c r="C8" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D8" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E8" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F8" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="G8">
         <v>7</v>
@@ -1284,19 +1328,19 @@
         <v>0</v>
       </c>
       <c r="L8" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="M8" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="N8" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="O8" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="T8" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
     </row>
     <row r="9" spans="1:20">
@@ -1307,16 +1351,16 @@
         <v>12</v>
       </c>
       <c r="C9" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E9" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F9" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="G9">
         <v>7</v>
@@ -1334,16 +1378,16 @@
         <v>0</v>
       </c>
       <c r="L9" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="M9" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="N9" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="O9" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="10" spans="1:20">
@@ -1354,13 +1398,13 @@
         <v>16</v>
       </c>
       <c r="C10" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D10" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E10" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G10">
         <v>3</v>
@@ -1378,16 +1422,19 @@
         <v>0</v>
       </c>
       <c r="L10" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="M10" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="N10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="O10" t="s">
-        <v>139</v>
+        <v>140</v>
+      </c>
+      <c r="T10" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="11" spans="1:20">
@@ -1398,16 +1445,16 @@
         <v>17</v>
       </c>
       <c r="C11" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D11" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E11" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F11" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G11">
         <v>3</v>
@@ -1425,16 +1472,19 @@
         <v>0</v>
       </c>
       <c r="L11" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="M11" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="N11" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="O11" t="s">
-        <v>140</v>
+        <v>141</v>
+      </c>
+      <c r="T11" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="12" spans="1:20">
@@ -1445,13 +1495,13 @@
         <v>18</v>
       </c>
       <c r="C12" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D12" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E12" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="G12">
         <v>3</v>
@@ -1469,16 +1519,19 @@
         <v>0</v>
       </c>
       <c r="L12" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="M12" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="N12" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="O12" t="s">
-        <v>141</v>
+        <v>142</v>
+      </c>
+      <c r="T12" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="13" spans="1:20">
@@ -1489,16 +1542,16 @@
         <v>19</v>
       </c>
       <c r="C13" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D13" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E13" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F13" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G13">
         <v>3</v>
@@ -1516,16 +1569,19 @@
         <v>0</v>
       </c>
       <c r="L13" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="M13" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="N13" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="O13" t="s">
-        <v>142</v>
+        <v>143</v>
+      </c>
+      <c r="T13" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="14" spans="1:20">
@@ -1536,13 +1592,13 @@
         <v>35</v>
       </c>
       <c r="C14" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D14" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E14" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G14">
         <v>1</v>
@@ -1560,16 +1616,19 @@
         <v>0</v>
       </c>
       <c r="L14" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="M14" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="N14" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="O14" t="s">
-        <v>143</v>
+        <v>144</v>
+      </c>
+      <c r="T14" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="15" spans="1:20">
@@ -1580,16 +1639,16 @@
         <v>36</v>
       </c>
       <c r="C15" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D15" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E15" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F15" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="G15">
         <v>1</v>
@@ -1607,19 +1666,19 @@
         <v>0</v>
       </c>
       <c r="L15" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="M15" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="N15" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="O15" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="T15" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
     </row>
     <row r="16" spans="1:20">
@@ -1630,16 +1689,16 @@
         <v>37</v>
       </c>
       <c r="C16" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D16" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E16" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F16" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="G16">
         <v>1</v>
@@ -1657,19 +1716,19 @@
         <v>0</v>
       </c>
       <c r="L16" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="M16" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="N16" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="O16" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="T16" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
     </row>
     <row r="17" spans="1:20">
@@ -1680,16 +1739,16 @@
         <v>38</v>
       </c>
       <c r="C17" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D17" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E17" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F17" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="G17">
         <v>1</v>
@@ -1707,19 +1766,19 @@
         <v>0</v>
       </c>
       <c r="L17" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="M17" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="N17" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="O17" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="T17" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
     </row>
     <row r="18" spans="1:20">
@@ -1730,16 +1789,16 @@
         <v>39</v>
       </c>
       <c r="C18" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D18" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E18" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F18" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="G18">
         <v>1</v>
@@ -1757,16 +1816,16 @@
         <v>0</v>
       </c>
       <c r="L18" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="M18" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="N18" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="O18" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="19" spans="1:20">
@@ -1777,13 +1836,13 @@
         <v>40</v>
       </c>
       <c r="C19" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D19" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E19" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="G19">
         <v>1</v>
@@ -1801,16 +1860,19 @@
         <v>0</v>
       </c>
       <c r="L19" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="M19" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="N19" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="O19" t="s">
-        <v>148</v>
+        <v>149</v>
+      </c>
+      <c r="T19" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="20" spans="1:20">
@@ -1821,13 +1883,13 @@
         <v>41</v>
       </c>
       <c r="C20" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D20" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E20" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="G20">
         <v>1</v>
@@ -1845,19 +1907,19 @@
         <v>0</v>
       </c>
       <c r="L20" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="M20" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="N20" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="O20" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="T20" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
     </row>
     <row r="21" spans="1:20">
@@ -1868,13 +1930,13 @@
         <v>42</v>
       </c>
       <c r="C21" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D21" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E21" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G21">
         <v>1</v>
@@ -1892,16 +1954,16 @@
         <v>0</v>
       </c>
       <c r="L21" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="M21" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="N21" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="O21" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="22" spans="1:20">
@@ -1912,16 +1974,16 @@
         <v>43</v>
       </c>
       <c r="C22" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D22" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E22" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F22" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="G22">
         <v>1</v>
@@ -1939,16 +2001,19 @@
         <v>0</v>
       </c>
       <c r="L22" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="M22" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="N22" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="O22" t="s">
-        <v>151</v>
+        <v>152</v>
+      </c>
+      <c r="T22" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="23" spans="1:20">
@@ -1959,13 +2024,13 @@
         <v>44</v>
       </c>
       <c r="C23" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D23" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E23" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G23">
         <v>1</v>
@@ -1983,19 +2048,19 @@
         <v>0</v>
       </c>
       <c r="L23" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="M23" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="N23" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="O23" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="T23" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
     </row>
     <row r="24" spans="1:20">
@@ -2006,16 +2071,16 @@
         <v>45</v>
       </c>
       <c r="C24" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D24" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E24" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F24" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="G24">
         <v>1</v>
@@ -2033,16 +2098,19 @@
         <v>0</v>
       </c>
       <c r="L24" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="M24" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="N24" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="O24" t="s">
-        <v>153</v>
+        <v>154</v>
+      </c>
+      <c r="T24" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="25" spans="1:20">
@@ -2053,13 +2121,13 @@
         <v>46</v>
       </c>
       <c r="C25" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D25" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E25" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="G25">
         <v>1</v>
@@ -2077,16 +2145,19 @@
         <v>0</v>
       </c>
       <c r="L25" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="M25" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="N25" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="O25" t="s">
-        <v>154</v>
+        <v>155</v>
+      </c>
+      <c r="T25" t="s">
+        <v>171</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Catalogue sprint: blind re-check of DSUK pilot (61/61 confirmed), 5 new advent pins, fan wikis classed as fan databases
Pilot now 100 pins / 23 official pages; reloads offline with all guards passing.
37 engine tests pass, audit clean.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EJKpUzadfBGAwYjvdRwUui
</commit_message>
<xml_diff>
--- a/docs/research/catalogue-sprint/pilot-dsuk-high/pilot_dsuk_high_checklist.xlsx
+++ b/docs/research/catalogue-sprint/pilot-dsuk-high/pilot_dsuk_high_checklist.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="166">
   <si>
     <t>Measure</t>
   </si>
@@ -110,6 +110,9 @@
     <t>dsuk/2025/ducks-of-disney-mystery-pouch</t>
   </si>
   <si>
+    <t>dsuk/2025/halloween-countdown-pin-advent-calendar</t>
+  </si>
+  <si>
     <t>dsuk/2025/pin-trading-25-years-mystery-set</t>
   </si>
   <si>
@@ -122,15 +125,9 @@
     <t>dsuk/2026/valentines-day-2026-mystery-set</t>
   </si>
   <si>
-    <t>dsuk/2024/muppets-haunted-mansion-mystery-puzzle-pin</t>
-  </si>
-  <si>
     <t>dsuk/2024/mickeys-christmas-carol-advent-calendar-2024</t>
   </si>
   <si>
-    <t>dsuk/2025/halloween-countdown-pin-advent-calendar</t>
-  </si>
-  <si>
     <t>dsuk/2025/celebrating-disney-pins-25-series-1</t>
   </si>
   <si>
@@ -179,6 +176,9 @@
     <t>Ducks of Disney Mystery Pin Pouch</t>
   </si>
   <si>
+    <t>Disney Halloween Limited Edition Countdown Pin Advent Calendar</t>
+  </si>
+  <si>
     <t>Disney Parks Pin Trading 25 Years Mystery Pin Set</t>
   </si>
   <si>
@@ -191,15 +191,9 @@
     <t>UK: Valentine's Day Limited Release Mystery Pin Set | AU: Disney Valentine's Day 2026 Mystery 2-Piece Pin Blind Pack</t>
   </si>
   <si>
-    <t>The Muppets Haunted Mansion Puzzle Piece Limited Edition Mystery Pin</t>
-  </si>
-  <si>
     <t>Mickey's Christmas Carol 24-Day Advent Calendar Mystery Pin Set 2024</t>
   </si>
   <si>
-    <t>Disney Halloween Limited Edition Countdown Pin Advent Calendar</t>
-  </si>
-  <si>
     <t>Celebrating Disney Pins 25th Anniversary Limited Edition Pin Set Series, 1 of 4</t>
   </si>
   <si>
@@ -248,15 +242,15 @@
     <t>2025-03-12</t>
   </si>
   <si>
+    <t>2025-07-28</t>
+  </si>
+  <si>
     <t>2025-05-22</t>
   </si>
   <si>
     <t>2024-09-30</t>
   </si>
   <si>
-    <t>2025-07-28</t>
-  </si>
-  <si>
     <t>2025-04-01</t>
   </si>
   <si>
@@ -281,6 +275,9 @@
     <t>https://www.disneystore.co.uk/ducks-of-disney-mystery-pin-pouch-438038208431.html</t>
   </si>
   <si>
+    <t>https://www.disneystore.eu/disney-halloween-limited-edition-countdown-pin-advent-calendar-438019866285.html</t>
+  </si>
+  <si>
     <t>https://www.disneystore.eu/disney-parks-pin-trading-25-years-mystery-pin-set-438019581485.html</t>
   </si>
   <si>
@@ -293,15 +290,9 @@
     <t>https://www.disneystore.co.uk/valentines-day-limited-release-mystery-pin-set-438010543840.html</t>
   </si>
   <si>
-    <t>https://www.disneystore.eu/the-muppets-haunted-mansion-puzzle-piece-limited-edition-mystery-pin-438017894693.html</t>
-  </si>
-  <si>
     <t>https://www.disneystore.eu/mickeys-christmas-carol-limited-edition-24-day-advent-calendar-mystery-pin-set-2024-438018036092.html</t>
   </si>
   <si>
-    <t>https://www.disneystore.co.uk/disney-halloween-limited-edition-countdown-pin-advent-calendar-438019866285.html</t>
-  </si>
-  <si>
     <t>https://www.disneystore.co.uk/celebrating-disney-pins-25th-anniversary-limited-edition-pin-set-series-1-of-4-438019714227.html</t>
   </si>
   <si>
@@ -353,6 +344,9 @@
     <t>Baymax – Ducks of Disney Mystery Pin Pouch | Cheshire Cat – Ducks of Disney Mystery Pin Pouch | Daisy Duck – Ducks of Disney Mystery Pin Pouch | Donald Duck – Ducks of Disney Mystery Pin Pouch | Dumbo – Ducks of Disney Mystery Pin Pouch | Figment – Ducks of Disney Mystery Pin Pouch | Goofy – Ducks of Disney Mystery Pin Pouch | Marie – Ducks of Disney Mystery Pin Pouch | Minnie Mouse – Ducks of Disney Mystery Pin Pouch | Nemo – Ducks of Disney Mystery Pin Pouch | Pluto – Ducks of Disney Mystery Pin Pouch | Powerline – Ducks of Disney Mystery Pin Pouch | Sorcerer Mickey – Ducks of Disney Mystery Pin Pouch | Stitch – Ducks of Disney Mystery Pin Pouch | Tigger – Ducks of Disney Mystery Pin Pouch | Tinker Bell – Ducks of Disney Mystery Pin Pouch</t>
   </si>
   <si>
+    <t>Chip – Disney Halloween Limited Edition Countdown Pin Advent Calendar | Daisy Duck – Disney Halloween Limited Edition Countdown Pin Advent Calendar | Dale – Disney Halloween Limited Edition Countdown Pin Advent Calendar | Donald Duck – Disney Halloween Limited Edition Countdown Pin Advent Calendar | Eeyore – Disney Halloween Limited Edition Countdown Pin Advent Calendar | Goofy – Disney Halloween Limited Edition Countdown Pin Advent Calendar | Max – Disney Halloween Limited Edition Countdown Pin Advent Calendar | Mickey Mouse – Disney Halloween Limited Edition Countdown Pin Advent Calendar | Minnie Mouse – Disney Halloween Limited Edition Countdown Pin Advent Calendar | Piglet – Disney Halloween Limited Edition Countdown Pin Advent Calendar | Pluto – Disney Halloween Limited Edition Countdown Pin Advent Calendar | Tigger – Disney Halloween Limited Edition Countdown Pin Advent Calendar | Winnie the Pooh – Disney Halloween Limited Edition Countdown Pin Advent Calendar</t>
+  </si>
+  <si>
     <t>Animal – Disney Parks Pin Trading 25 Years Mystery Pin Set | Baymax – Disney Parks Pin Trading 25 Years Mystery Pin Set | Donald Duck – Disney Parks Pin Trading 25 Years Mystery Pin Set | Genie – Disney Parks Pin Trading 25 Years Mystery Pin Set | Goofy – Disney Parks Pin Trading 25 Years Mystery Pin Set | Minnie Mouse – Disney Parks Pin Trading 25 Years Mystery Pin Set | Miss Piggy – Disney Parks Pin Trading 25 Years Mystery Pin Set | Pete – Disney Parks Pin Trading 25 Years Mystery Pin Set | Pluto – Disney Parks Pin Trading 25 Years Mystery Pin Set | Stitch – Disney Parks Pin Trading 25 Years Mystery Pin Set</t>
   </si>
   <si>
@@ -365,15 +359,9 @@
     <t>Baymax – UK: Valentine's Day Limited Release Mystery Pin Set | AU: Disney Valentine's Day 2026 Mystery 2-Piece Pin Blind Pack | Fozzie Bear – UK: Valentine's Day Limited Release Mystery Pin Set | AU: Disney Valentine's Day 2026 Mystery 2-Piece Pin Blind Pack | Genie – UK: Valentine's Day Limited Release Mystery Pin Set | AU: Disney Valentine's Day 2026 Mystery 2-Piece Pin Blind Pack | Hercules – UK: Valentine's Day Limited Release Mystery Pin Set | AU: Disney Valentine's Day 2026 Mystery 2-Piece Pin Blind Pack | Lucky – UK: Valentine's Day Limited Release Mystery Pin Set | AU: Disney Valentine's Day 2026 Mystery 2-Piece Pin Blind Pack | Mad Hatter – UK: Valentine's Day Limited Release Mystery Pin Set | AU: Disney Valentine's Day 2026 Mystery 2-Piece Pin Blind Pack | Marie – UK: Valentine's Day Limited Release Mystery Pin Set | AU: Disney Valentine's Day 2026 Mystery 2-Piece Pin Blind Pack | Powerline – UK: Valentine's Day Limited Release Mystery Pin Set | AU: Disney Valentine's Day 2026 Mystery 2-Piece Pin Blind Pack | Stitch – UK: Valentine's Day Limited Release Mystery Pin Set | AU: Disney Valentine's Day 2026 Mystery 2-Piece Pin Blind Pack | Winnie the Pooh – UK: Valentine's Day Limited Release Mystery Pin Set | AU: Disney Valentine's Day 2026 Mystery 2-Piece Pin Blind Pack</t>
   </si>
   <si>
-    <t>Dr. Bunsen Honeydew and Beaker as Busts | Chickens as Ghosts | The Electric Mayhem as Singing Ghosts | Fozzie as the Hatbox Ghost | Gonzo and Pepe as Servants | Haunted Mansion Exterior | Kermit and Miss Piggy in Mardi Gras costumes | Rowlf as Organist | Sam Eagle and Pops as Ghosts | Statler and Waldorf in a Doom Buggy</t>
-  </si>
-  <si>
     <t>Daisy Duck - Mickey's Christmas Carol Advent Calendar Pin | Donald Duck – Mickey's Christmas Carol 24-Day Advent Calendar Mystery Pin Set 2024 | Goofy - Mickey's Christmas Carol Advent Calendar Pin | Jiminy Cricket as The Ghost of Christmas Past | Mickey Mouse – Mickey's Christmas Carol 24-Day Advent Calendar Mystery Pin Set 2024 | Minnie Mouse - Mickey's Christmas Carol Advent Calendar Pin | Scrooge McDuck – Mickey's Christmas Carol 24-Day Advent Calendar Mystery Pin Set 2024</t>
   </si>
   <si>
-    <t>Chip – Disney Halloween Limited Edition Countdown Pin Advent Calendar | Daisy Duck – Disney Halloween Limited Edition Countdown Pin Advent Calendar | Eeyore – Disney Halloween Limited Edition Countdown Pin Advent Calendar | Max – Disney Halloween Limited Edition Countdown Pin Advent Calendar | Mickey Mouse – Disney Halloween Limited Edition Countdown Pin Advent Calendar | Pluto – Disney Halloween Limited Edition Countdown Pin Advent Calendar | Tigger – Disney Halloween Limited Edition Countdown Pin Advent Calendar</t>
-  </si>
-  <si>
     <t>Chip; Dale | Donald Duck – Celebrating Disney Pins 25th Anniversary Limited Edition Pin Set Series, 1 of 4 | Goofy – Celebrating Disney Pins 25th Anniversary Limited Edition Pin Set Series, 1 of 4</t>
   </si>
   <si>
@@ -416,6 +404,9 @@
     <t>dsuk/2025/ducks-of-disney-mystery-pouch/baymax | dsuk/2025/ducks-of-disney-mystery-pouch/cheshire-cat | dsuk/2025/ducks-of-disney-mystery-pouch/daisy | dsuk/2025/ducks-of-disney-mystery-pouch/donald | dsuk/2025/ducks-of-disney-mystery-pouch/dumbo | dsuk/2025/ducks-of-disney-mystery-pouch/figment | dsuk/2025/ducks-of-disney-mystery-pouch/goofy | dsuk/2025/ducks-of-disney-mystery-pouch/marie | dsuk/2025/ducks-of-disney-mystery-pouch/minnie | dsuk/2025/ducks-of-disney-mystery-pouch/nemo | dsuk/2025/ducks-of-disney-mystery-pouch/pluto | dsuk/2025/ducks-of-disney-mystery-pouch/powerline | dsuk/2025/ducks-of-disney-mystery-pouch/sorcerer-mickey | dsuk/2025/ducks-of-disney-mystery-pouch/stitch | dsuk/2025/ducks-of-disney-mystery-pouch/tigger | dsuk/2025/ducks-of-disney-mystery-pouch/tinker-bell</t>
   </si>
   <si>
+    <t>dsuk/2025/halloween-countdown-pin-advent-calendar/chip | dsuk/2025/halloween-countdown-pin-advent-calendar/daisy | dsuk/2025/halloween-countdown-pin-advent-calendar/dale | dsuk/2025/halloween-countdown-pin-advent-calendar/donald | dsuk/2025/halloween-countdown-pin-advent-calendar/eeyore | dsuk/2025/halloween-countdown-pin-advent-calendar/goofy | dsuk/2025/halloween-countdown-pin-advent-calendar/max | dsuk/2025/halloween-countdown-pin-advent-calendar/mickey | dsuk/2025/halloween-countdown-pin-advent-calendar/minnie | dsuk/2025/halloween-countdown-pin-advent-calendar/piglet | dsuk/2025/halloween-countdown-pin-advent-calendar/pluto | dsuk/2025/halloween-countdown-pin-advent-calendar/tigger | dsuk/2025/halloween-countdown-pin-advent-calendar/winnie-the-pooh</t>
+  </si>
+  <si>
     <t>dsuk/2025/pin-trading-25-years-mystery-set/animal | dsuk/2025/pin-trading-25-years-mystery-set/baymax | dsuk/2025/pin-trading-25-years-mystery-set/donald-duck | dsuk/2025/pin-trading-25-years-mystery-set/genie | dsuk/2025/pin-trading-25-years-mystery-set/goofy | dsuk/2025/pin-trading-25-years-mystery-set/minnie-mouse | dsuk/2025/pin-trading-25-years-mystery-set/miss-piggy | dsuk/2025/pin-trading-25-years-mystery-set/pete | dsuk/2025/pin-trading-25-years-mystery-set/pluto | dsuk/2025/pin-trading-25-years-mystery-set/stitch</t>
   </si>
   <si>
@@ -428,15 +419,9 @@
     <t>dsuk/2026/valentines-day-2026-mystery-set/baymax | dsuk/2026/valentines-day-2026-mystery-set/fozzie-bear | dsuk/2026/valentines-day-2026-mystery-set/genie | dsuk/2026/valentines-day-2026-mystery-set/hercules | dsuk/2026/valentines-day-2026-mystery-set/lucky | dsuk/2026/valentines-day-2026-mystery-set/mad-hatter | dsuk/2026/valentines-day-2026-mystery-set/marie | dsuk/2026/valentines-day-2026-mystery-set/powerline | dsuk/2026/valentines-day-2026-mystery-set/stitch | dsuk/2026/valentines-day-2026-mystery-set/winnie-the-pooh</t>
   </si>
   <si>
-    <t>dsuk/2024/muppets-haunted-mansion-mystery-puzzle-pin/bunsen-and-beaker-as-busts | dsuk/2024/muppets-haunted-mansion-mystery-puzzle-pin/chickens-as-ghosts | dsuk/2024/muppets-haunted-mansion-mystery-puzzle-pin/electric-mayhem-as-singing-ghosts | dsuk/2024/muppets-haunted-mansion-mystery-puzzle-pin/fozzie-as-hatbox-ghost | dsuk/2024/muppets-haunted-mansion-mystery-puzzle-pin/gonzo-and-pepe-as-servants | dsuk/2024/muppets-haunted-mansion-mystery-puzzle-pin/haunted-mansion-exterior | dsuk/2024/muppets-haunted-mansion-mystery-puzzle-pin/kermit-and-miss-piggy-mardi-gras | dsuk/2024/muppets-haunted-mansion-mystery-puzzle-pin/rowlf-as-organist | dsuk/2024/muppets-haunted-mansion-mystery-puzzle-pin/sam-eagle-and-pops-as-ghosts | dsuk/2024/muppets-haunted-mansion-mystery-puzzle-pin/statler-and-waldorf-doom-buggy</t>
-  </si>
-  <si>
     <t>dsuk/2024/mickeys-christmas-carol-advent-calendar-2024/daisy-isabelle | dsuk/2024/mickeys-christmas-carol-advent-calendar-2024/donald-fred | dsuk/2024/mickeys-christmas-carol-advent-calendar-2024/goofy-marleys-ghost | dsuk/2024/mickeys-christmas-carol-advent-calendar-2024/jiminy-cricket-ghost-of-christmas-past | dsuk/2024/mickeys-christmas-carol-advent-calendar-2024/mickey-bob-cratchit | dsuk/2024/mickeys-christmas-carol-advent-calendar-2024/minnie-emily-cratchit | dsuk/2024/mickeys-christmas-carol-advent-calendar-2024/scrooge-mcduck-ebenezer-scrooge</t>
   </si>
   <si>
-    <t>dsuk/2025/halloween-countdown-pin-advent-calendar/chip | dsuk/2025/halloween-countdown-pin-advent-calendar/daisy | dsuk/2025/halloween-countdown-pin-advent-calendar/eeyore | dsuk/2025/halloween-countdown-pin-advent-calendar/max | dsuk/2025/halloween-countdown-pin-advent-calendar/mickey | dsuk/2025/halloween-countdown-pin-advent-calendar/pluto | dsuk/2025/halloween-countdown-pin-advent-calendar/tigger</t>
-  </si>
-  <si>
     <t>dsuk/2025/celebrating-disney-pins-25-series-1/chip-n-dale | dsuk/2025/celebrating-disney-pins-25-series-1/donald-duck | dsuk/2025/celebrating-disney-pins-25-series-1/goofy</t>
   </si>
   <si>
@@ -489,9 +474,6 @@
   </si>
   <si>
     <t>powerline: possible duplicate; stitch: possible duplicate; winnie-the-pooh: possible duplicate</t>
-  </si>
-  <si>
-    <t>bunsen-and-beaker-as-busts: check one pin vs separate pins; gonzo-and-pepe-as-servants: check one pin vs separate pins; sam-eagle-and-pops-as-ghosts: check one pin vs separate pins</t>
   </si>
   <si>
     <t>daisy-isabelle: variants: add a note; donald-fred: variants: add a note; goofy-marleys-ghost: variants: add a note; jiminy-cricket-ghost-of-christmas-past: variants: add a note; mickey-bob-cratchit: variants: add a note; minnie-emily-cratchit: variants: add a note; scrooge-mcduck-ebenezer-scrooge: variants: add a note</t>
@@ -891,7 +873,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -931,7 +913,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -939,7 +921,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -949,7 +931,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T25"/>
+  <dimension ref="A1:T24"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:20">
@@ -1028,10 +1010,10 @@
         <v>30</v>
       </c>
       <c r="E2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="G2">
         <v>16</v>
@@ -1049,16 +1031,16 @@
         <v>0</v>
       </c>
       <c r="L2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="N2" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="O2" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
     </row>
     <row r="3" spans="1:20">
@@ -1066,7 +1048,7 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C3" t="s">
         <v>29</v>
@@ -1075,13 +1057,16 @@
         <v>31</v>
       </c>
       <c r="E3" t="s">
-        <v>54</v>
+        <v>53</v>
+      </c>
+      <c r="F3" t="s">
+        <v>75</v>
       </c>
       <c r="G3">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="H3">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="I3">
         <v>0</v>
@@ -1093,16 +1078,16 @@
         <v>0</v>
       </c>
       <c r="L3" t="s">
+        <v>84</v>
+      </c>
+      <c r="M3" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="M3" s="1" t="s">
-        <v>88</v>
-      </c>
       <c r="N3" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="O3" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
     </row>
     <row r="4" spans="1:20">
@@ -1119,10 +1104,7 @@
         <v>32</v>
       </c>
       <c r="E4" t="s">
-        <v>55</v>
-      </c>
-      <c r="F4" t="s">
-        <v>77</v>
+        <v>54</v>
       </c>
       <c r="G4">
         <v>10</v>
@@ -1140,16 +1122,16 @@
         <v>0</v>
       </c>
       <c r="L4" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="N4" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="O4" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
     </row>
     <row r="5" spans="1:20">
@@ -1166,7 +1148,10 @@
         <v>33</v>
       </c>
       <c r="E5" t="s">
-        <v>56</v>
+        <v>55</v>
+      </c>
+      <c r="F5" t="s">
+        <v>76</v>
       </c>
       <c r="G5">
         <v>10</v>
@@ -1184,19 +1169,16 @@
         <v>0</v>
       </c>
       <c r="L5" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M5" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="N5" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="O5" t="s">
-        <v>135</v>
-      </c>
-      <c r="T5" t="s">
-        <v>156</v>
+        <v>131</v>
       </c>
     </row>
     <row r="6" spans="1:20">
@@ -1213,7 +1195,7 @@
         <v>34</v>
       </c>
       <c r="E6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G6">
         <v>10</v>
@@ -1231,19 +1213,19 @@
         <v>0</v>
       </c>
       <c r="L6" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="N6" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="O6" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="T6" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
     </row>
     <row r="7" spans="1:20">
@@ -1260,16 +1242,16 @@
         <v>35</v>
       </c>
       <c r="E7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G7">
         <v>10</v>
       </c>
       <c r="H7">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="I7">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J7">
         <v>0</v>
@@ -1278,19 +1260,19 @@
         <v>0</v>
       </c>
       <c r="L7" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M7" s="1" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="N7" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="O7" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="T7" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
     </row>
     <row r="8" spans="1:20">
@@ -1298,7 +1280,7 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C8" t="s">
         <v>29</v>
@@ -1307,10 +1289,10 @@
         <v>36</v>
       </c>
       <c r="E8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G8">
         <v>7</v>
@@ -1328,19 +1310,19 @@
         <v>0</v>
       </c>
       <c r="L8" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M8" s="1" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="N8" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="O8" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="T8" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
     </row>
     <row r="9" spans="1:20">
@@ -1348,7 +1330,7 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C9" t="s">
         <v>29</v>
@@ -1357,16 +1339,13 @@
         <v>37</v>
       </c>
       <c r="E9" t="s">
-        <v>60</v>
-      </c>
-      <c r="F9" t="s">
-        <v>79</v>
+        <v>59</v>
       </c>
       <c r="G9">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="H9">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="I9">
         <v>0</v>
@@ -1378,16 +1357,19 @@
         <v>0</v>
       </c>
       <c r="L9" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M9" s="1" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="N9" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="O9" t="s">
-        <v>139</v>
+        <v>135</v>
+      </c>
+      <c r="T9" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="10" spans="1:20">
@@ -1395,7 +1377,7 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C10" t="s">
         <v>29</v>
@@ -1404,7 +1386,10 @@
         <v>38</v>
       </c>
       <c r="E10" t="s">
-        <v>61</v>
+        <v>60</v>
+      </c>
+      <c r="F10" t="s">
+        <v>78</v>
       </c>
       <c r="G10">
         <v>3</v>
@@ -1422,19 +1407,19 @@
         <v>0</v>
       </c>
       <c r="L10" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M10" s="1" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="N10" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="O10" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="T10" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
     </row>
     <row r="11" spans="1:20">
@@ -1442,7 +1427,7 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C11" t="s">
         <v>29</v>
@@ -1451,10 +1436,7 @@
         <v>39</v>
       </c>
       <c r="E11" t="s">
-        <v>62</v>
-      </c>
-      <c r="F11" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="G11">
         <v>3</v>
@@ -1472,19 +1454,19 @@
         <v>0</v>
       </c>
       <c r="L11" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M11" s="1" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="N11" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="O11" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="T11" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
     </row>
     <row r="12" spans="1:20">
@@ -1492,7 +1474,7 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C12" t="s">
         <v>29</v>
@@ -1501,7 +1483,10 @@
         <v>40</v>
       </c>
       <c r="E12" t="s">
-        <v>63</v>
+        <v>62</v>
+      </c>
+      <c r="F12" t="s">
+        <v>79</v>
       </c>
       <c r="G12">
         <v>3</v>
@@ -1519,19 +1504,19 @@
         <v>0</v>
       </c>
       <c r="L12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M12" s="1" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="N12" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="O12" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="T12" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
     </row>
     <row r="13" spans="1:20">
@@ -1539,7 +1524,7 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="C13" t="s">
         <v>29</v>
@@ -1548,16 +1533,13 @@
         <v>41</v>
       </c>
       <c r="E13" t="s">
-        <v>64</v>
-      </c>
-      <c r="F13" t="s">
-        <v>81</v>
+        <v>63</v>
       </c>
       <c r="G13">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H13">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I13">
         <v>0</v>
@@ -1569,19 +1551,19 @@
         <v>0</v>
       </c>
       <c r="L13" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M13" s="1" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="N13" t="s">
-        <v>122</v>
+        <v>63</v>
       </c>
       <c r="O13" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="T13" t="s">
-        <v>163</v>
+        <v>154</v>
       </c>
     </row>
     <row r="14" spans="1:20">
@@ -1589,7 +1571,7 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C14" t="s">
         <v>29</v>
@@ -1598,7 +1580,10 @@
         <v>42</v>
       </c>
       <c r="E14" t="s">
-        <v>65</v>
+        <v>64</v>
+      </c>
+      <c r="F14" t="s">
+        <v>80</v>
       </c>
       <c r="G14">
         <v>1</v>
@@ -1616,19 +1601,19 @@
         <v>0</v>
       </c>
       <c r="L14" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M14" s="1" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="N14" t="s">
-        <v>65</v>
+        <v>119</v>
       </c>
       <c r="O14" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="T14" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="15" spans="1:20">
@@ -1636,19 +1621,19 @@
         <v>14</v>
       </c>
       <c r="B15">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C15" t="s">
         <v>29</v>
       </c>
       <c r="D15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E15" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="F15" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G15">
         <v>1</v>
@@ -1666,19 +1651,19 @@
         <v>0</v>
       </c>
       <c r="L15" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M15" s="1" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="N15" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="O15" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="T15" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
     </row>
     <row r="16" spans="1:20">
@@ -1686,7 +1671,7 @@
         <v>15</v>
       </c>
       <c r="B16">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C16" t="s">
         <v>29</v>
@@ -1695,10 +1680,10 @@
         <v>43</v>
       </c>
       <c r="E16" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F16" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G16">
         <v>1</v>
@@ -1716,19 +1701,19 @@
         <v>0</v>
       </c>
       <c r="L16" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M16" s="1" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="N16" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="O16" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="T16" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
     </row>
     <row r="17" spans="1:20">
@@ -1736,7 +1721,7 @@
         <v>16</v>
       </c>
       <c r="B17">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C17" t="s">
         <v>29</v>
@@ -1745,10 +1730,10 @@
         <v>44</v>
       </c>
       <c r="E17" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F17" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="G17">
         <v>1</v>
@@ -1766,19 +1751,16 @@
         <v>0</v>
       </c>
       <c r="L17" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M17" s="1" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="N17" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="O17" t="s">
-        <v>147</v>
-      </c>
-      <c r="T17" t="s">
-        <v>166</v>
+        <v>143</v>
       </c>
     </row>
     <row r="18" spans="1:20">
@@ -1786,7 +1768,7 @@
         <v>17</v>
       </c>
       <c r="B18">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C18" t="s">
         <v>29</v>
@@ -1795,10 +1777,7 @@
         <v>45</v>
       </c>
       <c r="E18" t="s">
-        <v>68</v>
-      </c>
-      <c r="F18" t="s">
-        <v>82</v>
+        <v>67</v>
       </c>
       <c r="G18">
         <v>1</v>
@@ -1816,16 +1795,19 @@
         <v>0</v>
       </c>
       <c r="L18" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M18" s="1" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="N18" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="O18" t="s">
-        <v>148</v>
+        <v>144</v>
+      </c>
+      <c r="T18" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="19" spans="1:20">
@@ -1833,7 +1815,7 @@
         <v>18</v>
       </c>
       <c r="B19">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C19" t="s">
         <v>29</v>
@@ -1842,7 +1824,7 @@
         <v>46</v>
       </c>
       <c r="E19" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G19">
         <v>1</v>
@@ -1860,19 +1842,19 @@
         <v>0</v>
       </c>
       <c r="L19" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M19" s="1" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="N19" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="O19" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="T19" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
     </row>
     <row r="20" spans="1:20">
@@ -1880,7 +1862,7 @@
         <v>19</v>
       </c>
       <c r="B20">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C20" t="s">
         <v>29</v>
@@ -1889,7 +1871,7 @@
         <v>47</v>
       </c>
       <c r="E20" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G20">
         <v>1</v>
@@ -1907,19 +1889,16 @@
         <v>0</v>
       </c>
       <c r="L20" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M20" s="1" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="N20" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="O20" t="s">
-        <v>150</v>
-      </c>
-      <c r="T20" t="s">
-        <v>168</v>
+        <v>146</v>
       </c>
     </row>
     <row r="21" spans="1:20">
@@ -1927,7 +1906,7 @@
         <v>20</v>
       </c>
       <c r="B21">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C21" t="s">
         <v>29</v>
@@ -1936,7 +1915,10 @@
         <v>48</v>
       </c>
       <c r="E21" t="s">
-        <v>71</v>
+        <v>70</v>
+      </c>
+      <c r="F21" t="s">
+        <v>82</v>
       </c>
       <c r="G21">
         <v>1</v>
@@ -1954,16 +1936,19 @@
         <v>0</v>
       </c>
       <c r="L21" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M21" s="1" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="N21" t="s">
-        <v>129</v>
+        <v>70</v>
       </c>
       <c r="O21" t="s">
-        <v>151</v>
+        <v>147</v>
+      </c>
+      <c r="T21" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="22" spans="1:20">
@@ -1971,7 +1956,7 @@
         <v>21</v>
       </c>
       <c r="B22">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C22" t="s">
         <v>29</v>
@@ -1980,10 +1965,7 @@
         <v>49</v>
       </c>
       <c r="E22" t="s">
-        <v>72</v>
-      </c>
-      <c r="F22" t="s">
-        <v>84</v>
+        <v>71</v>
       </c>
       <c r="G22">
         <v>1</v>
@@ -2001,16 +1983,16 @@
         <v>0</v>
       </c>
       <c r="L22" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M22" s="1" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="N22" t="s">
-        <v>72</v>
+        <v>126</v>
       </c>
       <c r="O22" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="T22" t="s">
         <v>163</v>
@@ -2021,7 +2003,7 @@
         <v>22</v>
       </c>
       <c r="B23">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C23" t="s">
         <v>29</v>
@@ -2030,7 +2012,10 @@
         <v>50</v>
       </c>
       <c r="E23" t="s">
-        <v>73</v>
+        <v>72</v>
+      </c>
+      <c r="F23" t="s">
+        <v>83</v>
       </c>
       <c r="G23">
         <v>1</v>
@@ -2048,19 +2033,19 @@
         <v>0</v>
       </c>
       <c r="L23" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M23" s="1" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="N23" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="O23" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="T23" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
     </row>
     <row r="24" spans="1:20">
@@ -2068,7 +2053,7 @@
         <v>23</v>
       </c>
       <c r="B24">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C24" t="s">
         <v>29</v>
@@ -2077,10 +2062,7 @@
         <v>51</v>
       </c>
       <c r="E24" t="s">
-        <v>74</v>
-      </c>
-      <c r="F24" t="s">
-        <v>85</v>
+        <v>73</v>
       </c>
       <c r="G24">
         <v>1</v>
@@ -2098,66 +2080,19 @@
         <v>0</v>
       </c>
       <c r="L24" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M24" s="1" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="N24" t="s">
-        <v>131</v>
+        <v>73</v>
       </c>
       <c r="O24" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="T24" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="25" spans="1:20">
-      <c r="A25">
-        <v>24</v>
-      </c>
-      <c r="B25">
-        <v>46</v>
-      </c>
-      <c r="C25" t="s">
-        <v>29</v>
-      </c>
-      <c r="D25" t="s">
-        <v>52</v>
-      </c>
-      <c r="E25" t="s">
-        <v>75</v>
-      </c>
-      <c r="G25">
-        <v>1</v>
-      </c>
-      <c r="H25">
-        <v>1</v>
-      </c>
-      <c r="I25">
-        <v>0</v>
-      </c>
-      <c r="J25">
-        <v>0</v>
-      </c>
-      <c r="K25">
-        <v>0</v>
-      </c>
-      <c r="L25" t="s">
-        <v>86</v>
-      </c>
-      <c r="M25" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="N25" t="s">
-        <v>75</v>
-      </c>
-      <c r="O25" t="s">
-        <v>155</v>
-      </c>
-      <c r="T25" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
     </row>
   </sheetData>
@@ -2185,7 +2120,6 @@
     <hyperlink ref="M22" r:id="rId21"/>
     <hyperlink ref="M23" r:id="rId22"/>
     <hyperlink ref="M24" r:id="rId23"/>
-    <hyperlink ref="M25" r:id="rId24"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Catalogue sprint pass 6: disagreement and grouping-gap research; pilot refreshed
626 Day 2026 grouping confirmed by official listing (pilot structure checks 21 -> 11);
Goofy/Rafiki separate pins confirmed; 19 disagreements left for human review.
Pilot 100 pins / 23 pages / 700 evidence rows reloads offline. 44 tests pass, audit clean.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EJKpUzadfBGAwYjvdRwUui
</commit_message>
<xml_diff>
--- a/docs/research/catalogue-sprint/pilot-dsuk-high/pilot_dsuk_high_checklist.xlsx
+++ b/docs/research/catalogue-sprint/pilot-dsuk-high/pilot_dsuk_high_checklist.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="165">
   <si>
     <t>Measure</t>
   </si>
@@ -468,9 +468,6 @@
   </si>
   <si>
     <t>dsuk/2026/spider-man-hulk-brand-new-day-lr-pin/spider-man-and-hulk</t>
-  </si>
-  <si>
-    <t>627: check one pin vs separate pins; angel: check one pin vs separate pins; jumba: check one pin vs separate pins; kixx: check one pin vs separate pins; leroy: check one pin vs separate pins; reuben: check one pin vs separate pins; richter: check one pin vs separate pins; sinker: check one pin vs separate pins; splodyhead: check one pin vs separate pins; yaarp: check one pin vs separate pins</t>
   </si>
   <si>
     <t>powerline: possible duplicate; stitch: possible duplicate; winnie-the-pooh: possible duplicate</t>
@@ -913,7 +910,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>21</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -1224,9 +1221,6 @@
       <c r="O6" t="s">
         <v>132</v>
       </c>
-      <c r="T6" t="s">
-        <v>151</v>
-      </c>
     </row>
     <row r="7" spans="1:20">
       <c r="A7">
@@ -1272,7 +1266,7 @@
         <v>133</v>
       </c>
       <c r="T7" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="8" spans="1:20">
@@ -1322,7 +1316,7 @@
         <v>134</v>
       </c>
       <c r="T8" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="9" spans="1:20">
@@ -1369,7 +1363,7 @@
         <v>135</v>
       </c>
       <c r="T9" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="10" spans="1:20">
@@ -1419,7 +1413,7 @@
         <v>136</v>
       </c>
       <c r="T10" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="11" spans="1:20">
@@ -1466,7 +1460,7 @@
         <v>137</v>
       </c>
       <c r="T11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="12" spans="1:20">
@@ -1516,7 +1510,7 @@
         <v>138</v>
       </c>
       <c r="T12" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="13" spans="1:20">
@@ -1563,7 +1557,7 @@
         <v>139</v>
       </c>
       <c r="T13" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="14" spans="1:20">
@@ -1613,7 +1607,7 @@
         <v>140</v>
       </c>
       <c r="T14" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="15" spans="1:20">
@@ -1663,7 +1657,7 @@
         <v>141</v>
       </c>
       <c r="T15" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="16" spans="1:20">
@@ -1713,7 +1707,7 @@
         <v>142</v>
       </c>
       <c r="T16" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="17" spans="1:20">
@@ -1807,7 +1801,7 @@
         <v>144</v>
       </c>
       <c r="T18" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="19" spans="1:20">
@@ -1854,7 +1848,7 @@
         <v>145</v>
       </c>
       <c r="T19" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="20" spans="1:20">
@@ -1948,7 +1942,7 @@
         <v>147</v>
       </c>
       <c r="T21" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="22" spans="1:20">
@@ -1995,7 +1989,7 @@
         <v>148</v>
       </c>
       <c r="T22" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="23" spans="1:20">
@@ -2045,7 +2039,7 @@
         <v>149</v>
       </c>
       <c r="T23" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="24" spans="1:20">
@@ -2092,7 +2086,7 @@
         <v>150</v>
       </c>
       <c r="T24" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Catalogue sprint: evidence-based Brand/Release year for import; pilot dates; offline import replay (93/100 import)
- engine export: Brand from issuer or sale location (or official Disney Store listing),
  Release year from evidenced release date; title fallback uses characters
- 98_pilot_dates.json: set release dates/locations for 9 pilot sets
- tools/offline_import_test.mjs: real-schema replay of the #241 import (93 created,
  7 correctly refused; not public; linked; unique ids)
- laptop checklist: staging import steps

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EJKpUzadfBGAwYjvdRwUui
</commit_message>
<xml_diff>
--- a/docs/research/catalogue-sprint/pilot-dsuk-high/pilot_dsuk_high_checklist.xlsx
+++ b/docs/research/catalogue-sprint/pilot-dsuk-high/pilot_dsuk_high_checklist.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="172">
   <si>
     <t>Measure</t>
   </si>
@@ -248,12 +248,21 @@
     <t>2025-05-22</t>
   </si>
   <si>
+    <t>2026-06-30</t>
+  </si>
+  <si>
     <t>2024-09-30</t>
   </si>
   <si>
+    <t>2025-02-25</t>
+  </si>
+  <si>
     <t>2025-04-01</t>
   </si>
   <si>
+    <t>2025-09-02</t>
+  </si>
+  <si>
     <t>2025-10-08</t>
   </si>
   <si>
@@ -263,12 +272,18 @@
     <t>2023-12-12</t>
   </si>
   <si>
+    <t>2024-10-15</t>
+  </si>
+  <si>
     <t>2024-02</t>
   </si>
   <si>
     <t>2026-06-02</t>
   </si>
   <si>
+    <t>2026-07-07</t>
+  </si>
+  <si>
     <t>official</t>
   </si>
   <si>
@@ -353,7 +368,7 @@
     <t>Experiment 624 (Angel) | Experiment 010 (Felix) | Experiment 606 (Holio) | Experiment 604 (Houdini) | Experiment 629 (Leroy) | Experiment 625 (Reuben) | Experiment 221 (Sparky) | Experiment 619 (Splodyhead) | Experiment 626 (Stitch) | Experiment 502 (Yang)</t>
   </si>
   <si>
-    <t>627; Experiment 627; Stitch | Angel; Stitch | Jumba Jookiba; Stitch | Kixx; Stitch | Leroy; Stitch | Reuben; Stitch | Richter; Stitch | Sinker; Stitch | Splodyhead; Stitch | Stitch; Yaarp</t>
+    <t>627 &amp; Experiment 627 &amp; Stitch – Experiment 626 mystery pin set (626 Day 2026) | Angel &amp; Stitch – Experiment 626 mystery pin set (626 Day 2026) | Jumba Jookiba &amp; Stitch – Experiment 626 mystery pin set (626 Day 2026) | Kixx &amp; Stitch – Experiment 626 mystery pin set (626 Day 2026) | Leroy &amp; Stitch – Experiment 626 mystery pin set (626 Day 2026) | Reuben &amp; Stitch – Experiment 626 mystery pin set (626 Day 2026) | Richter &amp; Stitch – Experiment 626 mystery pin set (626 Day 2026) | Sinker &amp; Stitch – Experiment 626 mystery pin set (626 Day 2026) | Splodyhead &amp; Stitch – Experiment 626 mystery pin set (626 Day 2026) | Stitch &amp; Yaarp – Experiment 626 mystery pin set (626 Day 2026)</t>
   </si>
   <si>
     <t>Baymax – UK: Valentine's Day Limited Release Mystery Pin Set | AU: Disney Valentine's Day 2026 Mystery 2-Piece Pin Blind Pack | Fozzie Bear – UK: Valentine's Day Limited Release Mystery Pin Set | AU: Disney Valentine's Day 2026 Mystery 2-Piece Pin Blind Pack | Genie – UK: Valentine's Day Limited Release Mystery Pin Set | AU: Disney Valentine's Day 2026 Mystery 2-Piece Pin Blind Pack | Hercules – UK: Valentine's Day Limited Release Mystery Pin Set | AU: Disney Valentine's Day 2026 Mystery 2-Piece Pin Blind Pack | Lucky – UK: Valentine's Day Limited Release Mystery Pin Set | AU: Disney Valentine's Day 2026 Mystery 2-Piece Pin Blind Pack | Mad Hatter – UK: Valentine's Day Limited Release Mystery Pin Set | AU: Disney Valentine's Day 2026 Mystery 2-Piece Pin Blind Pack | Marie – UK: Valentine's Day Limited Release Mystery Pin Set | AU: Disney Valentine's Day 2026 Mystery 2-Piece Pin Blind Pack | Powerline – UK: Valentine's Day Limited Release Mystery Pin Set | AU: Disney Valentine's Day 2026 Mystery 2-Piece Pin Blind Pack | Stitch – UK: Valentine's Day Limited Release Mystery Pin Set | AU: Disney Valentine's Day 2026 Mystery 2-Piece Pin Blind Pack | Winnie the Pooh – UK: Valentine's Day Limited Release Mystery Pin Set | AU: Disney Valentine's Day 2026 Mystery 2-Piece Pin Blind Pack</t>
@@ -362,16 +377,16 @@
     <t>Daisy Duck - Mickey's Christmas Carol Advent Calendar Pin | Donald Duck – Mickey's Christmas Carol 24-Day Advent Calendar Mystery Pin Set 2024 | Goofy - Mickey's Christmas Carol Advent Calendar Pin | Jiminy Cricket as The Ghost of Christmas Past | Mickey Mouse – Mickey's Christmas Carol 24-Day Advent Calendar Mystery Pin Set 2024 | Minnie Mouse - Mickey's Christmas Carol Advent Calendar Pin | Scrooge McDuck – Mickey's Christmas Carol 24-Day Advent Calendar Mystery Pin Set 2024</t>
   </si>
   <si>
-    <t>Chip; Dale | Donald Duck – Celebrating Disney Pins 25th Anniversary Limited Edition Pin Set Series, 1 of 4 | Goofy – Celebrating Disney Pins 25th Anniversary Limited Edition Pin Set Series, 1 of 4</t>
-  </si>
-  <si>
-    <t>Jumba Jookiba – Celebrating Disney Pins 25th Anniversary Limited Edition Pin Set Series, 2 of 4 | Pleakley – Celebrating Disney Pins 25th Anniversary Limited Edition Pin Set Series, 2 of 4 | Angel; Stitch</t>
-  </si>
-  <si>
-    <t>Animal – Celebrating Disney Pins 25th Anniversary Limited Edition Pin Set Series, 3 of 4 | Fozzie Bear – Celebrating Disney Pins 25th Anniversary Limited Edition Pin Set Series, 3 of 4 | Kermit the Frog; Miss Piggy</t>
-  </si>
-  <si>
-    <t>Daisy Duck – Mickey and Friends Celebrating Disney Pins 25th Anniversary Limited Edition Pin Set Series, 4 of 4 | Mickey Mouse; Minnie Mouse | Pluto – Mickey and Friends Celebrating Disney Pins 25th Anniversary Limited Edition Pin Set Series, 4 of 4</t>
+    <t>Chip &amp; Dale – Celebrating Disney Pins 25th Anniversary Limited Edition Pin Set Series, 1 of 4 | Donald Duck – Celebrating Disney Pins 25th Anniversary Limited Edition Pin Set Series, 1 of 4 | Goofy – Celebrating Disney Pins 25th Anniversary Limited Edition Pin Set Series, 1 of 4</t>
+  </si>
+  <si>
+    <t>Jumba Jookiba – Celebrating Disney Pins 25th Anniversary Limited Edition Pin Set Series, 2 of 4 | Pleakley – Celebrating Disney Pins 25th Anniversary Limited Edition Pin Set Series, 2 of 4 | Angel &amp; Stitch – Celebrating Disney Pins 25th Anniversary Limited Edition Pin Set Series, 2 of 4</t>
+  </si>
+  <si>
+    <t>Animal – Celebrating Disney Pins 25th Anniversary Limited Edition Pin Set Series, 3 of 4 | Fozzie Bear – Celebrating Disney Pins 25th Anniversary Limited Edition Pin Set Series, 3 of 4 | Kermit the Frog &amp; Miss Piggy – Celebrating Disney Pins 25th Anniversary Limited Edition Pin Set Series, 3 of 4</t>
+  </si>
+  <si>
+    <t>Daisy Duck – Mickey and Friends Celebrating Disney Pins 25th Anniversary Limited Edition Pin Set Series, 4 of 4 | Mickey Mouse &amp; Minnie Mouse – Mickey and Friends Celebrating Disney Pins 25th Anniversary Limited Edition Pin Set Series, 4 of 4 | Pluto – Mickey and Friends Celebrating Disney Pins 25th Anniversary Limited Edition Pin Set Series, 4 of 4</t>
   </si>
   <si>
     <t>Belle and Chip Magical Collections Pin</t>
@@ -386,10 +401,10 @@
     <t>Big Hero 6 Magical Medallions Limited Release Pin</t>
   </si>
   <si>
-    <t>Mickey Mouse; Santa Claus</t>
-  </si>
-  <si>
-    <t>Hei Hei; Moana; Pua; Simea</t>
+    <t>Mickey Mouse &amp; Santa Claus – Mickey Mouse and Santa Claus Limited Release Festive Pin 2024</t>
+  </si>
+  <si>
+    <t>Hei Hei &amp; Moana &amp; Pua &amp; Simea – Moana, Simea, Pua and Hei Hei Limited Release Pin, Moana 2</t>
   </si>
   <si>
     <t>Mickey Mouse – Santa Mickey Mouse Limited Edition Festive Pin 2024</t>
@@ -398,7 +413,7 @@
     <t>Stitch St. Patrick's Day 2025 Limited Release Slider Pin, Lilo &amp; Stitch</t>
   </si>
   <si>
-    <t>Ariel; King Triton</t>
+    <t>Ariel &amp; King Triton – Ariel and King Triton Father's Day 2026 Limited Release Pin</t>
   </si>
   <si>
     <t>dsuk/2025/ducks-of-disney-mystery-pouch/baymax | dsuk/2025/ducks-of-disney-mystery-pouch/cheshire-cat | dsuk/2025/ducks-of-disney-mystery-pouch/daisy | dsuk/2025/ducks-of-disney-mystery-pouch/donald | dsuk/2025/ducks-of-disney-mystery-pouch/dumbo | dsuk/2025/ducks-of-disney-mystery-pouch/figment | dsuk/2025/ducks-of-disney-mystery-pouch/goofy | dsuk/2025/ducks-of-disney-mystery-pouch/marie | dsuk/2025/ducks-of-disney-mystery-pouch/minnie | dsuk/2025/ducks-of-disney-mystery-pouch/nemo | dsuk/2025/ducks-of-disney-mystery-pouch/pluto | dsuk/2025/ducks-of-disney-mystery-pouch/powerline | dsuk/2025/ducks-of-disney-mystery-pouch/sorcerer-mickey | dsuk/2025/ducks-of-disney-mystery-pouch/stitch | dsuk/2025/ducks-of-disney-mystery-pouch/tigger | dsuk/2025/ducks-of-disney-mystery-pouch/tinker-bell</t>
@@ -470,24 +485,30 @@
     <t>dsuk/2026/spider-man-hulk-brand-new-day-lr-pin/spider-man-and-hulk</t>
   </si>
   <si>
+    <t>stitch: possible duplicate</t>
+  </si>
+  <si>
     <t>powerline: possible duplicate; stitch: possible duplicate; winnie-the-pooh: possible duplicate</t>
   </si>
   <si>
     <t>daisy-isabelle: variants: add a note; donald-fred: variants: add a note; goofy-marleys-ghost: variants: add a note; jiminy-cricket-ghost-of-christmas-past: variants: add a note; mickey-bob-cratchit: variants: add a note; minnie-emily-cratchit: variants: add a note; scrooge-mcduck-ebenezer-scrooge: variants: add a note</t>
   </si>
   <si>
+    <t>chip-n-dale: variants: add a note, check one pin vs separate pins; donald-duck: variants: add a note; goofy: variants: add a note</t>
+  </si>
+  <si>
+    <t>stitch-with-angel: check one pin vs separate pins</t>
+  </si>
+  <si>
+    <t>animal: variants: add a note; fozzie: variants: add a note; kermit-and-miss-piggy: variants: add a note, check one pin vs separate pins</t>
+  </si>
+  <si>
+    <t>mickey-and-minnie: check one pin vs separate pins</t>
+  </si>
+  <si>
     <t>chip-n-dale: check one pin vs separate pins</t>
   </si>
   <si>
-    <t>stitch-with-angel: check one pin vs separate pins</t>
-  </si>
-  <si>
-    <t>kermit-and-miss-piggy: check one pin vs separate pins</t>
-  </si>
-  <si>
-    <t>mickey-and-minnie: check one pin vs separate pins</t>
-  </si>
-  <si>
     <t>belle-and-chip: variants: add a note, check one pin vs separate pins</t>
   </si>
   <si>
@@ -509,7 +530,7 @@
     <t>ariel-and-king-triton: check one pin vs separate pins</t>
   </si>
   <si>
-    <t>spider-man-and-hulk: check one pin vs separate pins</t>
+    <t>spider-man-and-hulk: variants: add a note, check one pin vs separate pins</t>
   </si>
 </sst>
 </file>
@@ -886,7 +907,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -894,7 +915,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>12</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -1028,16 +1049,16 @@
         <v>0</v>
       </c>
       <c r="L2" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="N2" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="O2" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
     </row>
     <row r="3" spans="1:20">
@@ -1075,16 +1096,16 @@
         <v>0</v>
       </c>
       <c r="L3" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="M3" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="N3" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="O3" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
     </row>
     <row r="4" spans="1:20">
@@ -1103,6 +1124,9 @@
       <c r="E4" t="s">
         <v>54</v>
       </c>
+      <c r="F4" t="s">
+        <v>76</v>
+      </c>
       <c r="G4">
         <v>10</v>
       </c>
@@ -1119,16 +1143,16 @@
         <v>0</v>
       </c>
       <c r="L4" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="N4" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="O4" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
     </row>
     <row r="5" spans="1:20">
@@ -1166,16 +1190,19 @@
         <v>0</v>
       </c>
       <c r="L5" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="M5" s="1" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="N5" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="O5" t="s">
-        <v>131</v>
+        <v>136</v>
+      </c>
+      <c r="T5" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="6" spans="1:20">
@@ -1194,6 +1221,9 @@
       <c r="E6" t="s">
         <v>56</v>
       </c>
+      <c r="F6" t="s">
+        <v>77</v>
+      </c>
       <c r="G6">
         <v>10</v>
       </c>
@@ -1210,16 +1240,16 @@
         <v>0</v>
       </c>
       <c r="L6" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="N6" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="O6" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
     </row>
     <row r="7" spans="1:20">
@@ -1254,19 +1284,19 @@
         <v>0</v>
       </c>
       <c r="L7" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="M7" s="1" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="N7" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="O7" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="T7" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
     </row>
     <row r="8" spans="1:20">
@@ -1286,7 +1316,7 @@
         <v>58</v>
       </c>
       <c r="F8" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="G8">
         <v>7</v>
@@ -1304,19 +1334,19 @@
         <v>0</v>
       </c>
       <c r="L8" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="M8" s="1" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="N8" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="O8" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="T8" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
     </row>
     <row r="9" spans="1:20">
@@ -1335,6 +1365,9 @@
       <c r="E9" t="s">
         <v>59</v>
       </c>
+      <c r="F9" t="s">
+        <v>79</v>
+      </c>
       <c r="G9">
         <v>3</v>
       </c>
@@ -1351,19 +1384,19 @@
         <v>0</v>
       </c>
       <c r="L9" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="M9" s="1" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="N9" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="O9" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="T9" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
     </row>
     <row r="10" spans="1:20">
@@ -1383,7 +1416,7 @@
         <v>60</v>
       </c>
       <c r="F10" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="G10">
         <v>3</v>
@@ -1401,19 +1434,19 @@
         <v>0</v>
       </c>
       <c r="L10" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="M10" s="1" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="N10" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="O10" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="T10" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
     </row>
     <row r="11" spans="1:20">
@@ -1432,6 +1465,9 @@
       <c r="E11" t="s">
         <v>61</v>
       </c>
+      <c r="F11" t="s">
+        <v>81</v>
+      </c>
       <c r="G11">
         <v>3</v>
       </c>
@@ -1448,19 +1484,19 @@
         <v>0</v>
       </c>
       <c r="L11" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="M11" s="1" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="N11" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="O11" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="T11" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
     </row>
     <row r="12" spans="1:20">
@@ -1480,7 +1516,7 @@
         <v>62</v>
       </c>
       <c r="F12" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="G12">
         <v>3</v>
@@ -1498,19 +1534,19 @@
         <v>0</v>
       </c>
       <c r="L12" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="M12" s="1" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="N12" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="O12" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="T12" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
     </row>
     <row r="13" spans="1:20">
@@ -1545,19 +1581,19 @@
         <v>0</v>
       </c>
       <c r="L13" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="M13" s="1" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="N13" t="s">
         <v>63</v>
       </c>
       <c r="O13" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="T13" t="s">
-        <v>153</v>
+        <v>163</v>
       </c>
     </row>
     <row r="14" spans="1:20">
@@ -1577,7 +1613,7 @@
         <v>64</v>
       </c>
       <c r="F14" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="G14">
         <v>1</v>
@@ -1595,19 +1631,19 @@
         <v>0</v>
       </c>
       <c r="L14" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="M14" s="1" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="N14" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="O14" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="T14" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
     </row>
     <row r="15" spans="1:20">
@@ -1627,7 +1663,7 @@
         <v>64</v>
       </c>
       <c r="F15" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="G15">
         <v>1</v>
@@ -1645,19 +1681,19 @@
         <v>0</v>
       </c>
       <c r="L15" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="M15" s="1" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="N15" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="O15" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="T15" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
     </row>
     <row r="16" spans="1:20">
@@ -1677,7 +1713,7 @@
         <v>65</v>
       </c>
       <c r="F16" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="G16">
         <v>1</v>
@@ -1695,19 +1731,19 @@
         <v>0</v>
       </c>
       <c r="L16" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="M16" s="1" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="N16" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="O16" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="T16" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
     </row>
     <row r="17" spans="1:20">
@@ -1727,7 +1763,7 @@
         <v>66</v>
       </c>
       <c r="F17" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="G17">
         <v>1</v>
@@ -1745,16 +1781,16 @@
         <v>0</v>
       </c>
       <c r="L17" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="M17" s="1" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="N17" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="O17" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
     </row>
     <row r="18" spans="1:20">
@@ -1773,6 +1809,9 @@
       <c r="E18" t="s">
         <v>67</v>
       </c>
+      <c r="F18" t="s">
+        <v>85</v>
+      </c>
       <c r="G18">
         <v>1</v>
       </c>
@@ -1789,19 +1828,19 @@
         <v>0</v>
       </c>
       <c r="L18" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="M18" s="1" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="N18" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="O18" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="T18" t="s">
-        <v>160</v>
+        <v>167</v>
       </c>
     </row>
     <row r="19" spans="1:20">
@@ -1836,19 +1875,19 @@
         <v>0</v>
       </c>
       <c r="L19" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="M19" s="1" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="N19" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="O19" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="T19" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
     </row>
     <row r="20" spans="1:20">
@@ -1883,16 +1922,16 @@
         <v>0</v>
       </c>
       <c r="L20" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="M20" s="1" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="N20" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="O20" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
     </row>
     <row r="21" spans="1:20">
@@ -1912,7 +1951,7 @@
         <v>70</v>
       </c>
       <c r="F21" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="G21">
         <v>1</v>
@@ -1930,19 +1969,19 @@
         <v>0</v>
       </c>
       <c r="L21" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="M21" s="1" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="N21" t="s">
         <v>70</v>
       </c>
       <c r="O21" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="T21" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
     </row>
     <row r="22" spans="1:20">
@@ -1977,19 +2016,19 @@
         <v>0</v>
       </c>
       <c r="L22" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="M22" s="1" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="N22" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="O22" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="T22" t="s">
-        <v>162</v>
+        <v>169</v>
       </c>
     </row>
     <row r="23" spans="1:20">
@@ -2009,7 +2048,7 @@
         <v>72</v>
       </c>
       <c r="F23" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="G23">
         <v>1</v>
@@ -2027,19 +2066,19 @@
         <v>0</v>
       </c>
       <c r="L23" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="M23" s="1" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="N23" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="O23" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="T23" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
     </row>
     <row r="24" spans="1:20">
@@ -2058,6 +2097,9 @@
       <c r="E24" t="s">
         <v>73</v>
       </c>
+      <c r="F24" t="s">
+        <v>88</v>
+      </c>
       <c r="G24">
         <v>1</v>
       </c>
@@ -2074,19 +2116,19 @@
         <v>0</v>
       </c>
       <c r="L24" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="M24" s="1" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="N24" t="s">
         <v>73</v>
       </c>
       <c r="O24" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="T24" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
     </row>
   </sheetData>

</xml_diff>